<commit_message>
Correct eight points in Confidence Intervals for Proportions and Differences
An interval that excludes 0 makes the difference statistically distinguishable from zero, which the page now says in place of "truly differ" and "real". It matches the next part's tests exactly only with the same unpooled standard error, the formula assumes independent groups (a shared test set calls for a paired method), and the lift's interval is [+0.7, +6.6]. The notebook figure's title no longer says B sits clearly above A, the margin of error is the half-width, the A/B data is a realistic teaching set, and the codebook's ID pattern has seven characters.
</commit_message>
<xml_diff>
--- a/data/confidence-intervals-for-proportions-and-differences--ab_test.xlsx
+++ b/data/confidence-intervals-for-proportions-and-differences--ab_test.xlsx
@@ -60530,7 +60530,7 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Vxxxxx</t>
+          <t>Vxxxxxx</t>
         </is>
       </c>
     </row>
@@ -60671,7 +60671,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>WHAT IS CAPTURED: a randomized A/B test log, one row per visitor.</t>
+          <t>WHAT IS CAPTURED: a randomized A/B test log, one row per visitor (a realistic teaching dataset written for the book).</t>
         </is>
       </c>
     </row>

</xml_diff>